<commit_message>
Antes de cambiar la interfaz
</commit_message>
<xml_diff>
--- a/src/main/java/com/mycompany/ocxrst/BASES/INTORDENDECOMPRA.xlsx
+++ b/src/main/java/com/mycompany/ocxrst/BASES/INTORDENDECOMPRA.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\OCXRST\OrdendeComprasRST\src\main\java\com\mycompany\ocxrst\BASES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1469F88E-8890-4A4B-8C45-328973A14366}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28715A0-6E48-45E3-8C06-4DD9B861EEF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3024" yWindow="2304" windowWidth="16740" windowHeight="9372" xr2:uid="{92F47CF0-95F9-4D84-814C-7AFFA20164B6}"/>
+    <workbookView xWindow="612" yWindow="-108" windowWidth="22536" windowHeight="13176" xr2:uid="{92F47CF0-95F9-4D84-814C-7AFFA20164B6}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$I$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$I$52</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="44">
   <si>
     <t>CODIGO</t>
   </si>
@@ -57,15 +57,54 @@
     <t>PENDIENTE_RECIBIR</t>
   </si>
   <si>
+    <t>MOU8200</t>
+  </si>
+  <si>
+    <t>Mouse óptico inalámbrico de tres botones con sensor de alta precisión, diseño compacto y receptor USB para equipos de escritorio y portátiles</t>
+  </si>
+  <si>
+    <t>PZA</t>
+  </si>
+  <si>
+    <t>PAPBOND75</t>
+  </si>
+  <si>
+    <t>Papel bond blanco tamaño carta de 75 gramos, paquete de alta blancura para impresión y copiado cotidiano de documentos administrativos</t>
+  </si>
+  <si>
+    <t>PAQ</t>
+  </si>
+  <si>
+    <t>REG1200</t>
+  </si>
+  <si>
+    <t>Regulador electrónico de voltaje de 1200 VA con protección contra variaciones eléctricas y múltiples contactos para equipos de cómputo</t>
+  </si>
+  <si>
+    <t>LIMP500</t>
+  </si>
+  <si>
+    <t>Limpiador líquido multiusos de 500 ml para superficies de oficina, formulado para remover polvo, grasa ligera y suciedad cotidiana</t>
+  </si>
+  <si>
+    <t>EXT6-10M</t>
+  </si>
+  <si>
+    <t>Extensión eléctrica de 10 metros con cable reforzado, clavija polarizada y contactos múltiples para conectar equipos y accesorios en áreas de trabajo</t>
+  </si>
+  <si>
+    <t>W2300A</t>
+  </si>
+  <si>
+    <t>Tóner original W2300A Negro</t>
+  </si>
+  <si>
     <t>W2301A</t>
   </si>
   <si>
     <t>Tóner original W2300A Cian</t>
   </si>
   <si>
-    <t>PZA</t>
-  </si>
-  <si>
     <t>W2302A</t>
   </si>
   <si>
@@ -84,37 +123,43 @@
     <t>Papel bond tamaño carta 75g</t>
   </si>
   <si>
-    <t>PAQ</t>
-  </si>
-  <si>
     <t>HP1021</t>
   </si>
   <si>
     <t>Papel bond tamaño oficio 75g</t>
   </si>
   <si>
+    <t>CAN002</t>
+  </si>
+  <si>
+    <t>Cartucho Canon PG-210 Negro</t>
+  </si>
+  <si>
+    <t>EPSON01</t>
+  </si>
+  <si>
+    <t>Tinta Epson 544 Negro</t>
+  </si>
+  <si>
+    <t>ML</t>
+  </si>
+  <si>
+    <t>EPSON02</t>
+  </si>
+  <si>
+    <t>Tinta Epson 544 Cian</t>
+  </si>
+  <si>
+    <t>EPSON03</t>
+  </si>
+  <si>
+    <t>Tinta Epson 544 Magenta</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
     <t>0</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>W2300A</t>
-  </si>
-  <si>
-    <t>Tóner original W2300A Negro</t>
   </si>
 </sst>
 </file>
@@ -493,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1658ADDC-DCFD-4FC0-A51D-94B360144F05}">
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" bestFit="true" customWidth="true" width="12.44140625" collapsed="true"/>
@@ -547,16 +592,16 @@
         <v>1.0</v>
       </c>
       <c r="F2" t="n">
-        <v>2137.51</v>
+        <v>289.5</v>
       </c>
       <c r="G2" t="n">
-        <v>2137.51</v>
+        <v>289.5</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3">
@@ -570,22 +615,22 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E3" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="F3" t="n">
-        <v>2137.51</v>
+        <v>118.6</v>
       </c>
       <c r="G3" t="n">
-        <v>4275.02</v>
+        <v>118.6</v>
       </c>
       <c r="H3" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="I3" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4">
@@ -593,28 +638,28 @@
         <v>1.0</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
       </c>
       <c r="E4" t="n">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
       <c r="F4" t="n">
-        <v>2137.51</v>
+        <v>895.25</v>
       </c>
       <c r="G4" t="n">
-        <v>12825.060000000001</v>
+        <v>895.25</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -622,28 +667,28 @@
         <v>1.0</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E5" t="n">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="F5" t="n">
-        <v>95.5</v>
+        <v>86.9</v>
       </c>
       <c r="G5" t="n">
-        <v>382.0</v>
+        <v>86.9</v>
       </c>
       <c r="H5" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="I5" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6">
@@ -657,33 +702,33 @@
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E6" t="n">
         <v>1.0</v>
       </c>
       <c r="F6" t="n">
-        <v>110.25</v>
+        <v>349.9</v>
       </c>
       <c r="G6" t="n">
-        <v>110.25</v>
+        <v>349.9</v>
       </c>
       <c r="H6" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="I6" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
@@ -692,172 +737,172 @@
         <v>1.0</v>
       </c>
       <c r="F7" t="n">
-        <v>2137.51</v>
+        <v>1771.62</v>
       </c>
       <c r="G7" t="n">
-        <v>2137.51</v>
+        <v>1771.62</v>
       </c>
       <c r="H7" t="s">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="I7" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
         <v>11</v>
       </c>
       <c r="E8" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="F8" t="n">
         <v>2137.51</v>
       </c>
       <c r="G8" t="n">
-        <v>4275.02</v>
+        <v>2137.51</v>
       </c>
       <c r="H8" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="I8" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D9" t="s">
         <v>11</v>
       </c>
       <c r="E9" t="n">
-        <v>6.0</v>
+        <v>1.0</v>
       </c>
       <c r="F9" t="n">
         <v>2137.51</v>
       </c>
       <c r="G9" t="n">
-        <v>12825.060000000001</v>
+        <v>2137.51</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="I9" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E10" t="n">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="F10" t="n">
-        <v>95.5</v>
+        <v>2137.51</v>
       </c>
       <c r="G10" t="n">
-        <v>382.0</v>
+        <v>2137.51</v>
       </c>
       <c r="H10" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="I10" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E11" t="n">
         <v>1.0</v>
       </c>
       <c r="F11" t="n">
-        <v>110.25</v>
+        <v>95.5</v>
       </c>
       <c r="G11" t="n">
-        <v>110.25</v>
+        <v>95.5</v>
       </c>
       <c r="H11" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="I11" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E12" t="n">
         <v>1.0</v>
       </c>
       <c r="F12" t="n">
-        <v>1771.62</v>
+        <v>110.25</v>
       </c>
       <c r="G12" t="n">
-        <v>1771.62</v>
+        <v>110.25</v>
       </c>
       <c r="H12" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="I12" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="B13" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="D13" t="s">
         <v>11</v>
@@ -866,80 +911,385 @@
         <v>1.0</v>
       </c>
       <c r="F13" t="n">
-        <v>2137.51</v>
+        <v>580.0</v>
       </c>
       <c r="G13" t="n">
-        <v>2137.51</v>
+        <v>580.0</v>
       </c>
       <c r="H13" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="I13" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>37</v>
       </c>
       <c r="E14" t="n">
         <v>1.0</v>
       </c>
       <c r="F14" t="n">
-        <v>2137.51</v>
+        <v>210.75</v>
       </c>
       <c r="G14" t="n">
-        <v>2137.51</v>
+        <v>210.75</v>
       </c>
       <c r="H14" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="I14" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>205.6</v>
+      </c>
+      <c r="G15" t="n">
+        <v>205.6</v>
+      </c>
+      <c r="H15" t="s">
+        <v>43</v>
+      </c>
+      <c r="I15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="B16" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>205.6</v>
+      </c>
+      <c r="G16" t="n">
+        <v>205.6</v>
+      </c>
+      <c r="H16" t="s">
+        <v>43</v>
+      </c>
+      <c r="I16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" t="s">
         <v>14</v>
       </c>
-      <c r="C15" t="s">
+      <c r="E17" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>118.6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>118.6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B18" t="s">
         <v>15</v>
       </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="F15" t="n">
+      <c r="C18" t="s">
+        <v>16</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>895.25</v>
+      </c>
+      <c r="G18" t="n">
+        <v>895.25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B19" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>86.9</v>
+      </c>
+      <c r="G19" t="n">
+        <v>86.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>349.9</v>
+      </c>
+      <c r="G20" t="n">
+        <v>349.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D21" t="s">
+        <v>11</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1771.62</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1771.62</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F22" t="n">
         <v>2137.51</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G22" t="n">
         <v>2137.51</v>
       </c>
-      <c r="H15" t="s">
-        <v>21</v>
-      </c>
-      <c r="I15" t="s">
-        <v>22</v>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2137.51</v>
+      </c>
+      <c r="G24" t="n">
+        <v>2137.51</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>29</v>
+      </c>
+      <c r="C25" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" t="n">
+        <v>100.0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>95.5</v>
+      </c>
+      <c r="G25" t="n">
+        <v>9550.0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B26" t="s">
+        <v>33</v>
+      </c>
+      <c r="C26" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>580.0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>580.0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B27" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" t="s">
+        <v>37</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>210.75</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1053.75</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C28" t="s">
+        <v>41</v>
+      </c>
+      <c r="D28" t="s">
+        <v>37</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>205.6</v>
+      </c>
+      <c r="G28" t="n">
+        <v>205.6</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I80" xr:uid="{7D811ECF-302C-4453-AA90-921548F2E119}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I80">
-      <sortCondition ref="A1:A80"/>
+  <autoFilter ref="A1:I52" xr:uid="{7D811ECF-302C-4453-AA90-921548F2E119}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I52">
+      <sortCondition ref="A1:A52"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>